<commit_message>
Add feature classifier pipeline, field-photo preprocess, and scan UI.
Two-stage inference (class ~88%, features ~70%), field photo ETL scripts, installation-aware preprocessing, search/export fixes, and geometric scan preview. Remove legacy MNIST artifacts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/templates/markup_template.xlsx
+++ b/data/templates/markup_template.xlsx
@@ -7,7 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="объект 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="кельты" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ножи" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="удила" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="наконечники стрел" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="накладки" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,27 +433,226 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>признак 1</t>
+          <t>материал</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>признак 2</t>
+          <t>сохранность</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>признак 3</t>
+          <t>форма</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>признак 4</t>
+          <t>тулья</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>признак 5</t>
+          <t>ушки</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>номер</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>название</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>материал</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>сохранность</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>тип</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>рукоять</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>орнамент</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>номер</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>название</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>материал</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>сохранность</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>тип_окончания</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>шарнирность</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>номер</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>название</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>материал</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>сохранность</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>тип_насадки</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>форма_лезвия</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>сечение</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>номер</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>название</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>материал</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>сохранность</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>форма</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>крепление</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>орнамент</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix camera capture black frames; normalize tables; update training/eval pipeline
- Improve Windows camera capture reliability (warmup, backend fallback, black-frame rejection)
- Add table normalization utilities/scripts and refresh templates/models
- Update training/evaluation and scan UI wiring

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/templates/markup_template.xlsx
+++ b/data/templates/markup_template.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="кельты" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ножи" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="удила" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="наконечники стрел" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="накладки" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="кельты" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ножи" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="удила" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="наконечники стрел" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="накладки" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -591,12 +591,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>тип_насадки</t>
+          <t>тип_насада</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>форма_лезвия</t>
+          <t>форма_пера</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">

</xml_diff>